<commit_message>
work on referral task
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" state="visible" r:id="rId2"/>
@@ -171,8 +171,8 @@
     <t xml:space="preserve">intro</t>
   </si>
   <si>
-    <t xml:space="preserve">SAY: I’m coming to check up on you. On my visit on {last_visit_date}, I gave you a referral to the health facility for the following reasons:
-{referral_reasons}</t>
+    <t xml:space="preserve">SAY: I’m coming to check up on you. On my visit on ${last_visit_date}, I gave you a referral to the health facility for the following reasons:
+${referral_reasons}</t>
   </si>
   <si>
     <t xml:space="preserve">select_one yes_no</t>

</xml_diff>

<commit_message>
change form and task to have task reasons in form
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="129">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -81,6 +81,9 @@
     <t xml:space="preserve">inputs</t>
   </si>
   <si>
+    <t xml:space="preserve">NO_LABEL</t>
+  </si>
+  <si>
     <t xml:space="preserve">hidden</t>
   </si>
   <si>
@@ -90,7 +93,25 @@
     <t xml:space="preserve">last_visit_date</t>
   </si>
   <si>
-    <t xml:space="preserve">referral_reasons</t>
+    <t xml:space="preserve">refer_flag_small_baby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_neonatal_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_child_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_muac_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_palm_pallor_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_vaccines_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refer_slow_to_learn_specifics_flag</t>
   </si>
   <si>
     <t xml:space="preserve">user</t>
@@ -135,6 +156,33 @@
     <t xml:space="preserve">calculate</t>
   </si>
   <si>
+    <t xml:space="preserve">last_visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/last_visit_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_flag_small_baby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_neonatal_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_child_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_muac_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_refer_palm_pallor_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_vaccines_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../inputs/refer_slow_to_learn_specifics_flag</t>
+  </si>
+  <si>
     <t xml:space="preserve">client</t>
   </si>
   <si>
@@ -147,18 +195,6 @@
     <t xml:space="preserve">../inputs/contact/name</t>
   </si>
   <si>
-    <t xml:space="preserve">last_visit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../inputs/last_visit_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reasons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../inputs/reasons</t>
-  </si>
-  <si>
     <t xml:space="preserve">referral_follow_up</t>
   </si>
   <si>
@@ -171,8 +207,70 @@
     <t xml:space="preserve">intro</t>
   </si>
   <si>
-    <t xml:space="preserve">SAY: I’m coming to check up on you. On my visit on ${last_visit_date}, I gave you a referral to the health facility for the following reasons:
-${referral_reasons}</t>
+    <t xml:space="preserve">SAY: I’m coming to check up on you. On my visit on ${last_visit_date}, I gave you a referral to the health facility for the following reasons:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_flag_small_baby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small baby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../refer_flag_small_baby = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_neonatal_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neonatal danger sign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_neonatal_danger_sign_flag = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_child_danger_sign_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Child danger sign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_child_danger_sign_flag = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_muac_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_muac_flag = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_palm_pallor_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palm pallor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_refer_palm_pallor_flag = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_vaccines_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vaccines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_vaccines_flag = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason_refer_slow_to_learn_specifics_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slow learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/refer_slow_to_learn_specifics_flag = 1</t>
   </si>
   <si>
     <t xml:space="preserve">select_one yes_no</t>
@@ -393,13 +491,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -431,7 +533,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="1" style="0" width="14.43"/>
@@ -497,121 +599,148 @@
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C2" s="0" t="s">
+        <v>19</v>
+      </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1" t="s">
         <v>25</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>27</v>
+      <c r="C7" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>30</v>
@@ -619,219 +748,452 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>40</v>
+        <v>1</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L19" s="2" t="s">
-        <v>42</v>
+      <c r="C19" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>56</v>
+        <v>43</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" s="0" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>56</v>
+        <v>24</v>
+      </c>
+      <c r="L25" s="0" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
+      </c>
+      <c r="L26" s="0" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C27" s="3"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1" t="s">
-        <v>63</v>
+        <v>26</v>
+      </c>
+      <c r="L27" s="0" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>53</v>
+        <v>27</v>
+      </c>
+      <c r="L28" s="0" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>68</v>
+        <v>28</v>
+      </c>
+      <c r="L29" s="0" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>53</v>
+        <v>29</v>
+      </c>
+      <c r="L30" s="0" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>73</v>
+        <v>53</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
+        <v>57</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F35" s="0" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F39" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -856,7 +1218,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -870,74 +1232,74 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -964,32 +1326,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>43584</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Referral resolved if (#7)
* add source id and source form to form
* include translations into referral_form
* carry over referral flags for referral_follow_up form
* fix resolvedIf for referral_follow_up task
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heix\Documents\GitHub\config-dtree\forms\app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Heiko Hornung\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB06BAD3-3CA6-46A7-A7CB-F9DEB2D9C744}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
     <sheet name="choices" sheetId="2" r:id="rId2"/>
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="159">
   <si>
     <t>type</t>
   </si>
@@ -95,6 +94,12 @@
     <t>string</t>
   </si>
   <si>
+    <t>source_form</t>
+  </si>
+  <si>
+    <t>source_id</t>
+  </si>
+  <si>
     <t>last_visit_date</t>
   </si>
   <si>
@@ -161,6 +166,24 @@
     <t>calculate</t>
   </si>
   <si>
+    <t>patient_id</t>
+  </si>
+  <si>
+    <t>../inputs/contact/_id</t>
+  </si>
+  <si>
+    <t>referral_source_form</t>
+  </si>
+  <si>
+    <t>../inputs/source_form</t>
+  </si>
+  <si>
+    <t>referral_source_id</t>
+  </si>
+  <si>
+    <t>../inputs/source_id</t>
+  </si>
+  <si>
     <t>last_visit</t>
   </si>
   <si>
@@ -191,9 +214,6 @@
     <t>client</t>
   </si>
   <si>
-    <t>../inputs/contact/_id</t>
-  </si>
-  <si>
     <t>client_name</t>
   </si>
   <si>
@@ -350,6 +370,15 @@
     <t>selected(${complete_referral},"yes")</t>
   </si>
   <si>
+    <t>has_referral</t>
+  </si>
+  <si>
+    <t>if(selected(${complete_referral},"yes"),1,0)</t>
+  </si>
+  <si>
+    <t>referral_days</t>
+  </si>
+  <si>
     <t>list_name</t>
   </si>
   <si>
@@ -416,20 +445,71 @@
     <t>Referral Follow-up</t>
   </si>
   <si>
-    <t>has_referral</t>
-  </si>
-  <si>
-    <t>if(selected(${complete_referral},"yes"),1,0)</t>
-  </si>
-  <si>
-    <t>referral_days</t>
+    <t>Sina pesa</t>
+  </si>
+  <si>
+    <t>Sikutaka kwenda</t>
+  </si>
+  <si>
+    <t>Sikupewa ruhusa ya kwenda</t>
+  </si>
+  <si>
+    <t>Nyenginezo</t>
+  </si>
+  <si>
+    <t>Ufuasi wa rufaa</t>
+  </si>
+  <si>
+    <t>SEMA: Nimekuja kukuangalia. Wakati nilipokutemebela mara ya mwisho nilikupa rufaa ya kuenda kituo cha afya kutokana na sababu zifuatazo:</t>
+  </si>
+  <si>
+    <t>Mtoto Njiti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dalili za hatari kwa mtoto baada ya kuzaliwa </t>
+  </si>
+  <si>
+    <t>Dalili za hatari kwa mtoto</t>
+  </si>
+  <si>
+    <t>Viganja viko vyeupe sana</t>
+  </si>
+  <si>
+    <t>Chanjo</t>
+  </si>
+  <si>
+    <t>Mzito kujifunza</t>
+  </si>
+  <si>
+    <t>ULIZA: Je ulienda kituo cha afya?</t>
+  </si>
+  <si>
+    <t>Mpongeze mteja kwa kuenda kituo cha afya</t>
+  </si>
+  <si>
+    <t>ULIZA: Je ulipata huduma?</t>
+  </si>
+  <si>
+    <t>Jadili sababu na jaribu kutatua tatizo na panga naye kuhusu kukamilisha rufaa</t>
+  </si>
+  <si>
+    <t>ULIZA: Kwa nini hukwenda kituo cha afya?</t>
+  </si>
+  <si>
+    <t>Jadili sababu na jaribu kumpa ushauri wa jinsi ya kutatua tatizo na panga naye njia ya yeye kupata huduma</t>
+  </si>
+  <si>
+    <t>ULIZA: Je unafikiri unahitaji kuikamilisha rufaa hii?</t>
+  </si>
+  <si>
+    <t>Nitarudi baba ya siku 3 ili kuhakikisha kuwa umekamilisha hii rufaa.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -438,6 +518,11 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Arial"/>
       <charset val="1"/>
     </font>
@@ -462,17 +547,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,7 +591,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -519,7 +603,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -566,23 +650,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -618,23 +685,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -786,11 +836,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q59"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1025" width="14.42578125" customWidth="1"/>
+    <col min="1" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="4" width="14.42578125" style="6" customWidth="1"/>
+    <col min="5" max="1025" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -853,7 +905,7 @@
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -867,20 +919,22 @@
       <c r="B3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>19</v>
       </c>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>19</v>
       </c>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -889,7 +943,7 @@
       <c r="B5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -897,10 +951,10 @@
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -911,7 +965,7 @@
       <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -922,7 +976,7 @@
       <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -933,7 +987,7 @@
       <c r="B9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -944,18 +998,18 @@
       <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -966,19 +1020,19 @@
       <c r="B12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>32</v>
+      <c r="C12" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -986,29 +1040,32 @@
         <v>21</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="C16" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1016,35 +1073,32 @@
         <v>38</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="6" t="s">
         <v>19</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1052,431 +1106,538 @@
         <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>44</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L24" t="s">
-        <v>46</v>
+        <v>38</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L25" t="s">
+        <v>46</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="L26" t="s">
         <v>48</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="L27" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L28" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>28</v>
+        <v>45</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="L29" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="L30" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>54</v>
+        <v>27</v>
+      </c>
+      <c r="L31" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+      <c r="L32" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L33" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L35" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="B38" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B36" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="D38" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F36" t="s">
+      <c r="B39" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="D39" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F37" t="s">
+      <c r="C40" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B38" s="1" t="s">
+      <c r="D40" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F40" t="s">
         <v>71</v>
       </c>
-      <c r="C38" s="4" t="s">
+    </row>
+    <row r="41" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F38" t="s">
+      <c r="C41" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="D41" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F41" t="s">
         <v>74</v>
       </c>
-      <c r="C39" s="4" t="s">
+    </row>
+    <row r="42" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F39" t="s">
+      <c r="C42" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="1" t="s">
+      <c r="D42" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F42" t="s">
         <v>77</v>
       </c>
-      <c r="C40" s="4" t="s">
+    </row>
+    <row r="43" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F40" t="s">
+      <c r="C43" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B41" s="1" t="s">
+      <c r="D43" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="4" t="s">
+    </row>
+    <row r="44" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F41" t="s">
+      <c r="C44" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="D44" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F44" t="s">
         <v>83</v>
       </c>
-      <c r="B42" s="1" t="s">
+    </row>
+    <row r="45" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="D45" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F45" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="1" t="s">
+    <row r="46" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C46" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="D46" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F46" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B44" s="1" t="s">
+    <row r="47" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="B47" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B45" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="D47" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F45" s="1" t="s">
+    </row>
+    <row r="48" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C46" t="s">
-        <v>19</v>
-      </c>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1" t="s">
+      <c r="D48" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F48" s="1" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>36</v>
+        <v>104</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>43</v>
-      </c>
-      <c r="B53" t="s">
-        <v>129</v>
-      </c>
-      <c r="L53" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="L54">
+        <v>109</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>45</v>
+      </c>
+      <c r="B58" t="s">
+        <v>114</v>
+      </c>
+      <c r="L58" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="L59">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1485,7 +1646,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1499,74 +1660,86 @@
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
+      </c>
+      <c r="D4" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>117</v>
+        <v>127</v>
+      </c>
+      <c r="D5" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
+      </c>
+      <c r="D6" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>121</v>
+        <v>131</v>
+      </c>
+      <c r="D7" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1576,7 +1749,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1585,30 +1758,30 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C2" s="5">
         <v>43584</v>

</xml_diff>

<commit_message>
Added a referral follow-up for a woman who is 6 months pregnant or mo… (#97)
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="281">
   <si>
     <t>type</t>
   </si>
@@ -144,6 +144,9 @@
     <t>refer_flag_postpartum_other_signs</t>
   </si>
   <si>
+    <t>refer_flag_anc_visit_6m_or_more</t>
+  </si>
+  <si>
     <t>user</t>
   </si>
   <si>
@@ -204,6 +207,12 @@
     <t>../inputs/original_source_form</t>
   </si>
   <si>
+    <t>form_title</t>
+  </si>
+  <si>
+    <t>list_name</t>
+  </si>
+  <si>
     <t>referral_source_id</t>
   </si>
   <si>
@@ -216,21 +225,48 @@
     <t>../inputs/last_visit_date</t>
   </si>
   <si>
+    <t>form_id</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>instance_name</t>
+  </si>
+  <si>
+    <t>Referral Follow-up</t>
+  </si>
+  <si>
     <t>last_visit_formatted</t>
   </si>
   <si>
+    <t>referral_follow_up</t>
+  </si>
+  <si>
     <t>format-date-time(../inputs/last_visit_date div (1000*60*60*24), "%d/%m/%Y")</t>
   </si>
   <si>
     <t>../inputs/refer_flag_small_baby</t>
   </si>
   <si>
+    <t>pages</t>
+  </si>
+  <si>
     <t>../inputs/refer_neonatal_danger_sign_flag</t>
   </si>
   <si>
     <t>../inputs/refer_secondary_neonatal_danger_sign_flag</t>
   </si>
   <si>
+    <t>data</t>
+  </si>
+  <si>
     <t>../inputs/refer_child_danger_sign_flag</t>
   </si>
   <si>
@@ -240,69 +276,147 @@
     <t>../inputs/refer_refer_palm_pallor_flag</t>
   </si>
   <si>
+    <t>yes_no</t>
+  </si>
+  <si>
     <t>../inputs/refer_vaccines_flag</t>
   </si>
   <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Ndiyo</t>
+  </si>
+  <si>
     <t>../inputs/refer_slow_to_learn_specifics_flag</t>
   </si>
   <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Hapana</t>
+  </si>
+  <si>
     <t>client</t>
   </si>
   <si>
+    <t>reason_didnt_go</t>
+  </si>
+  <si>
+    <t>no_money</t>
+  </si>
+  <si>
+    <t>I have no money</t>
+  </si>
+  <si>
     <t>client_name</t>
   </si>
   <si>
+    <t>Sina pesa</t>
+  </si>
+  <si>
     <t>../inputs/contact/name</t>
   </si>
   <si>
+    <t>did_not_want</t>
+  </si>
+  <si>
+    <t>I did not want to go</t>
+  </si>
+  <si>
     <t>client_date_of_birth</t>
   </si>
   <si>
-    <t>form_title</t>
-  </si>
-  <si>
-    <t>form_id</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>instance_name</t>
-  </si>
-  <si>
-    <t>Referral Follow-up</t>
-  </si>
-  <si>
-    <t>referral_follow_up</t>
+    <t>Sikutaka kwenda</t>
+  </si>
+  <si>
+    <t>no_permission</t>
+  </si>
+  <si>
+    <t>I did not have permission to go</t>
+  </si>
+  <si>
+    <t>Sikupewa ruhusa ya kwenda</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Nyenginezo</t>
+  </si>
+  <si>
+    <t>reason_didnt_get_svc</t>
+  </si>
+  <si>
+    <t>too_many_people</t>
+  </si>
+  <si>
+    <t>There were too many people</t>
+  </si>
+  <si>
+    <t>Kulikuwa na watu wengi</t>
   </si>
   <si>
     <t>../inputs/contact/date_of_birth</t>
   </si>
   <si>
-    <t>pages</t>
+    <t>services_not_offered</t>
+  </si>
+  <si>
+    <t>The services I needed were not offered when I went</t>
+  </si>
+  <si>
+    <t>Huduma nilizotaka hazikuwepo.</t>
   </si>
   <si>
     <t>../inputs/due_date</t>
   </si>
   <si>
+    <t>no_service_provider_available</t>
+  </si>
+  <si>
+    <t>No service providers were available</t>
+  </si>
+  <si>
+    <t>Hakukuwa na mtoa huduma</t>
+  </si>
+  <si>
     <t>due_date_pretty_print</t>
   </si>
   <si>
-    <t>data</t>
-  </si>
-  <si>
     <t>../inputs/due_date_human_readable</t>
   </si>
   <si>
+    <t>was_asked_to_pay</t>
+  </si>
+  <si>
+    <t>I was asked to pay for services</t>
+  </si>
+  <si>
+    <t>Walitaka nilipie huduma</t>
+  </si>
+  <si>
     <t>../inputs/refer_flag_emergency_danger_sign</t>
   </si>
   <si>
+    <t>was_treated_badly</t>
+  </si>
+  <si>
+    <t>Health workers treated me badly</t>
+  </si>
+  <si>
+    <t>Wahudumu wa afya hawakunihudumia vizuri</t>
+  </si>
+  <si>
     <t>../inputs/refer_flag_pregnancy_issues</t>
   </si>
   <si>
@@ -315,6 +429,9 @@
     <t>../inputs/refer_flag_postpartum_other_signs</t>
   </si>
   <si>
+    <t>../inputs/refer_flag_anc_visit_6m_or_more</t>
+  </si>
+  <si>
     <t>age_days</t>
   </si>
   <si>
@@ -328,117 +445,6 @@
   </si>
   <si>
     <t>age_years</t>
-  </si>
-  <si>
-    <t>list_name</t>
-  </si>
-  <si>
-    <t>yes_no</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Ndiyo</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Hapana</t>
-  </si>
-  <si>
-    <t>reason_didnt_go</t>
-  </si>
-  <si>
-    <t>no_money</t>
-  </si>
-  <si>
-    <t>I have no money</t>
-  </si>
-  <si>
-    <t>Sina pesa</t>
-  </si>
-  <si>
-    <t>did_not_want</t>
-  </si>
-  <si>
-    <t>I did not want to go</t>
-  </si>
-  <si>
-    <t>Sikutaka kwenda</t>
-  </si>
-  <si>
-    <t>no_permission</t>
-  </si>
-  <si>
-    <t>I did not have permission to go</t>
-  </si>
-  <si>
-    <t>Sikupewa ruhusa ya kwenda</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Nyenginezo</t>
-  </si>
-  <si>
-    <t>reason_didnt_get_svc</t>
-  </si>
-  <si>
-    <t>too_many_people</t>
-  </si>
-  <si>
-    <t>There were too many people</t>
-  </si>
-  <si>
-    <t>Kulikuwa na watu wengi</t>
-  </si>
-  <si>
-    <t>services_not_offered</t>
-  </si>
-  <si>
-    <t>The services I needed were not offered when I went</t>
-  </si>
-  <si>
-    <t>Huduma nilizotaka hazikuwepo.</t>
-  </si>
-  <si>
-    <t>no_service_provider_available</t>
-  </si>
-  <si>
-    <t>No service providers were available</t>
-  </si>
-  <si>
-    <t>Hakukuwa na mtoa huduma</t>
-  </si>
-  <si>
-    <t>was_asked_to_pay</t>
-  </si>
-  <si>
-    <t>I was asked to pay for services</t>
-  </si>
-  <si>
-    <t>Walitaka nilipie huduma</t>
-  </si>
-  <si>
-    <t>was_treated_badly</t>
-  </si>
-  <si>
-    <t>Health workers treated me badly</t>
-  </si>
-  <si>
-    <t>Wahudumu wa afya hawakunihudumia vizuri</t>
   </si>
   <si>
     <t>int(${age_days} div (30 *12),0)</t>
@@ -693,6 +699,18 @@
     <t>../../inputs/refer_flag_postpartum_other_signs= 1</t>
   </si>
   <si>
+    <t>reason_refer_flag_anc_visit_6m_or_more</t>
+  </si>
+  <si>
+    <t>&lt;span style="display:block;padding-left:1em"&gt;To get ANC services since your pregnancy is 6 months or more.&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style="display:block;padding-left:1em"&gt;Ili kupatiwa huduma za mama mjamzito kwa vile mimba yako ni miezi sita au zaidi.&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>../../inputs/refer_flag_anc_visit_6m_or_more= 1</t>
+  </si>
+  <si>
     <t>select_one yes_no</t>
   </si>
   <si>
@@ -831,7 +849,7 @@
     <t>has_pregnancy_referral</t>
   </si>
   <si>
-    <t xml:space="preserve">../inputs/refer_flag_emergency_danger_sign  = 1 or ../inputs/refer_flag_pregnancy_issues  = 1 or  ../inputs/refer_flag_pregnancy_complications = 1 </t>
+    <t>../inputs/refer_flag_emergency_danger_sign  = 1 or ../inputs/refer_flag_pregnancy_issues  = 1 or  ../inputs/refer_flag_pregnancy_complications = 1 or ../inputs/refer_flag_anc_visit_6m_or_more = 1</t>
   </si>
   <si>
     <t>has_infant_child_referral</t>
@@ -865,10 +883,10 @@
       <name val="Roboto"/>
     </font>
     <font>
+      <sz val="10.0"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -910,16 +928,16 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -928,7 +946,7 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1277,26 +1295,26 @@
       <c r="D21" s="1"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="1" t="s">
+      <c r="A22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="1"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D23" s="1"/>
     </row>
@@ -1305,10 +1323,10 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="D24" s="1"/>
     </row>
@@ -1317,7 +1335,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>48</v>
@@ -1326,59 +1344,59 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="1"/>
       <c r="D26" s="1"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="C27" s="1"/>
       <c r="D27" s="1"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D28" s="1"/>
-      <c r="G28" s="1" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="1"/>
+      <c r="G29" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>19</v>
@@ -1399,1113 +1417,1144 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" s="1"/>
+        <v>56</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="D32" s="1"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
-      <c r="L34" s="1" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="L35" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
-      <c r="L36" s="3" t="s">
+      <c r="L36" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
-      <c r="L37" s="1" t="s">
-        <v>64</v>
+      <c r="L37" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="L38" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>67</v>
+      <c r="A39" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
-      <c r="L39" s="4" t="s">
-        <v>68</v>
+      <c r="L39" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>28</v>
+      <c r="A40" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
-      <c r="L40" t="s">
-        <v>69</v>
+      <c r="L40" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>29</v>
+        <v>57</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="L41" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
-      <c r="L42" s="3" t="s">
-        <v>71</v>
+      <c r="L42" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
-      <c r="L43" t="s">
-        <v>72</v>
+      <c r="L43" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="L44" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="L45" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
       <c r="L46" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="L47" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
-      <c r="L48" s="1" t="s">
-        <v>58</v>
+      <c r="L48" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C50" s="5"/>
-      <c r="D50" s="7"/>
-      <c r="L50" s="3" t="s">
-        <v>89</v>
+      <c r="A50" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="L50" s="1" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="C51" s="8"/>
+      <c r="D51" s="9"/>
       <c r="L51" s="3" t="s">
-        <v>91</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="9"/>
       <c r="L52" s="3" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="7"/>
-      <c r="L53" s="10" t="s">
-        <v>95</v>
+        <v>125</v>
+      </c>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="L53" s="3" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C54" s="5"/>
-      <c r="D54" s="7"/>
+        <v>38</v>
+      </c>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
       <c r="L54" s="10" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C55" s="5"/>
-      <c r="D55" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
       <c r="L55" s="10" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="D56" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="C56" s="8"/>
+      <c r="D56" s="9"/>
       <c r="L56" s="10" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="7"/>
+        <v>41</v>
+      </c>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
       <c r="L57" s="10" t="s">
-        <v>99</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="7"/>
-      <c r="L58" s="11" t="s">
-        <v>101</v>
+        <v>42</v>
+      </c>
+      <c r="C58" s="8"/>
+      <c r="D58" s="9"/>
+      <c r="L58" s="10" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="7"/>
-      <c r="L59" s="12" t="s">
-        <v>103</v>
+        <v>43</v>
+      </c>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="L59" s="10" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C60" s="5"/>
-      <c r="D60" s="7"/>
-      <c r="L60" s="12" t="s">
-        <v>142</v>
+        <v>139</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="L60" s="11" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B61" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="7"/>
+        <v>57</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C61" s="8"/>
+      <c r="D61" s="9"/>
       <c r="L61" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B62" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="7"/>
-      <c r="L62" s="15" t="s">
-        <v>146</v>
+        <v>57</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="L62" s="12" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B63" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="7"/>
-      <c r="L63" s="15" t="s">
-        <v>148</v>
+        <v>57</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C63" s="8"/>
+      <c r="D63" s="9"/>
+      <c r="L63" s="12" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="7"/>
+        <v>147</v>
+      </c>
+      <c r="C64" s="8"/>
+      <c r="D64" s="9"/>
       <c r="L64" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
       <c r="L65" s="15" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D66" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>156</v>
+        <v>57</v>
+      </c>
+      <c r="B66" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="L66" s="15" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>160</v>
+        <v>57</v>
+      </c>
+      <c r="B67" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="L67" s="15" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D68" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B68" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>163</v>
+      <c r="G68" s="3" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="3" t="s">
-        <v>49</v>
+        <v>159</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C71" s="1"/>
-      <c r="D71" s="4"/>
+        <v>166</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C72" s="1" t="s">
+      <c r="A72" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C72" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D72" s="4" t="s">
+      <c r="D72" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G72" s="3" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>174</v>
-      </c>
+      <c r="A73" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C73" s="1"/>
+      <c r="D73" s="5"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="1" t="s">
-        <v>157</v>
+        <v>17</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>175</v>
+        <v>77</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="F74" s="3" t="s">
-        <v>178</v>
+        <v>172</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="A76" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D76" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="F76" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="F75" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B77" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F77" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="78" ht="15.75" customHeight="1">
+      <c r="A78" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="F78" s="3" t="s">
         <v>188</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F77" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F78" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>191</v>
       </c>
       <c r="F79" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>201</v>
+        <v>193</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>195</v>
       </c>
       <c r="F80" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="F81" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="F82" t="s">
         <v>204</v>
       </c>
-      <c r="D81" s="4" t="s">
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="F81" t="s">
+      <c r="C83" s="5" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B82" s="3" t="s">
+      <c r="D83" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="F83" t="s">
         <v>208</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="E82" s="1"/>
-      <c r="F82" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E83" s="1"/>
-      <c r="F83" s="3" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>217</v>
+        <v>210</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>211</v>
       </c>
       <c r="E84" s="1"/>
-      <c r="F84" s="3" t="s">
-        <v>218</v>
+      <c r="F84" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>215</v>
       </c>
       <c r="E85" s="1"/>
       <c r="F85" s="3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E86" s="1"/>
+      <c r="F86" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C87" s="2" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="1" t="s">
+      <c r="D87" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="E87" s="1"/>
+      <c r="F87" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C86" s="4" t="s">
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B88" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D86" s="4" t="s">
+      <c r="C88" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B87" s="4" t="s">
+      <c r="D88" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C87" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D87" s="1"/>
-      <c r="E87" s="1"/>
-      <c r="F87" s="1" t="s">
+      <c r="E88" s="1"/>
+      <c r="F88" s="2" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="F88" s="1"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="1" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B89" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D89" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="E89" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="90" ht="15.75" customHeight="1">
+      <c r="A90" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B90" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D89" s="4" t="s">
+      <c r="C90" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="F89" s="1"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C90" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="D90" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="E90" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F90" s="4" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B91" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" ht="15.75" customHeight="1">
+      <c r="A92" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="D92" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="E92" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" ht="15.75" customHeight="1">
+      <c r="A93" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D91" s="4" t="s">
+      <c r="B93" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="F91" s="4" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="C92" s="1"/>
-      <c r="D92" s="1"/>
-      <c r="E92" s="1"/>
-      <c r="F92" s="1"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B93" s="1" t="s">
+      <c r="C93" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="C93" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D93" s="1"/>
-      <c r="E93" s="1"/>
-      <c r="F93" s="1" t="s">
+      <c r="D93" s="5" t="s">
         <v>244</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="F94" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C94" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="D94" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="D95" s="4" t="s">
-        <v>250</v>
-      </c>
+      <c r="A95" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="1" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="C96" s="1"/>
+        <v>249</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="D96" s="1"/>
       <c r="E96" s="1"/>
+      <c r="F96" s="1" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B97" s="4" t="s">
+      <c r="A97" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="C97" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D97" s="1"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="4" t="s">
+      <c r="B97" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C97" s="5" t="s">
         <v>252</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="1" t="s">
-        <v>223</v>
+        <v>159</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="C98" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="D98" s="4" t="s">
+      <c r="C98" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="E98" s="1" t="s">
-        <v>107</v>
+      <c r="D98" s="5" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="C99" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+    </row>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B100" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D99" s="1" t="s">
+      <c r="C100" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="F99" s="1" t="s">
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B100" s="4" t="s">
+      <c r="C101" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="C100" s="4"/>
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
-      <c r="L100" s="4" t="s">
+      <c r="D101" s="5" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B101" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="C101" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="D101" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="E101" s="4"/>
-      <c r="F101" t="s">
-        <v>265</v>
+      <c r="E101" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="C102" s="1"/>
-      <c r="D102" s="1"/>
+        <v>159</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C103" s="1"/>
-      <c r="D103" s="1"/>
-    </row>
-    <row r="104" ht="12.75" customHeight="1">
-      <c r="A104" t="s">
-        <v>56</v>
-      </c>
-      <c r="B104" s="3" t="s">
+      <c r="A103" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B103" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="C104" s="1"/>
-      <c r="D104" s="1"/>
-      <c r="L104" t="s">
+      <c r="C103" s="5"/>
+      <c r="D103" s="5"/>
+      <c r="E103" s="5"/>
+      <c r="L103" s="5" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="105" ht="12.75" customHeight="1">
-      <c r="A105" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B105" s="3" t="s">
+    <row r="104" ht="15.75" customHeight="1">
+      <c r="A104" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B104" s="5" t="s">
         <v>268</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="E104" s="5"/>
+      <c r="F104" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="105" ht="15.75" customHeight="1">
+      <c r="A105" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>257</v>
       </c>
       <c r="C105" s="1"/>
       <c r="D105" s="1"/>
-      <c r="L105" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="106" ht="12.75" customHeight="1">
-      <c r="A106" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>270</v>
+    </row>
+    <row r="106" ht="15.75" customHeight="1">
+      <c r="A106" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>77</v>
       </c>
       <c r="C106" s="1"/>
       <c r="D106" s="1"/>
-      <c r="L106" s="2" t="s">
-        <v>271</v>
-      </c>
     </row>
     <row r="107" ht="12.75" customHeight="1">
-      <c r="A107" s="3" t="s">
-        <v>56</v>
+      <c r="A107" t="s">
+        <v>57</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>272</v>
       </c>
       <c r="C107" s="1"/>
       <c r="D107" s="1"/>
-      <c r="L107" s="3" t="s">
+      <c r="L107" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="108" ht="12.75" customHeight="1">
-      <c r="A108" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B108" s="1" t="s">
+      <c r="A108" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B108" s="3" t="s">
         <v>274</v>
       </c>
       <c r="C108" s="1"/>
       <c r="D108" s="1"/>
-      <c r="L108">
-        <v>3.0</v>
+      <c r="L108" s="3" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="109" ht="12.75" customHeight="1">
+      <c r="A109" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="C109" s="1"/>
       <c r="D109" s="1"/>
+      <c r="L109" s="2" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="110" ht="12.75" customHeight="1">
+      <c r="A110" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="C110" s="1"/>
       <c r="D110" s="1"/>
+      <c r="L110" s="3" t="s">
+        <v>279</v>
+      </c>
     </row>
     <row r="111" ht="12.75" customHeight="1">
+      <c r="A111" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>280</v>
+      </c>
       <c r="C111" s="1"/>
       <c r="D111" s="1"/>
+      <c r="L111">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="112" ht="12.75" customHeight="1">
       <c r="C112" s="1"/>
@@ -6258,6 +6307,18 @@
     <row r="1049" ht="12.75" customHeight="1">
       <c r="C1049" s="1"/>
       <c r="D1049" s="1"/>
+    </row>
+    <row r="1050" ht="12.75" customHeight="1">
+      <c r="C1050" s="1"/>
+      <c r="D1050" s="1"/>
+    </row>
+    <row r="1051" ht="12.75" customHeight="1">
+      <c r="C1051" s="1"/>
+      <c r="D1051" s="1"/>
+    </row>
+    <row r="1052" ht="12.75" customHeight="1">
+      <c r="C1052" s="1"/>
+      <c r="D1052" s="1"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -6281,185 +6342,185 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="6" t="s">
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D7" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1"/>
@@ -7471,40 +7532,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>86</v>
+      <c r="A1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="8">
+        <v>77</v>
+      </c>
+      <c r="C2" s="6">
         <v>43584.0</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>93</v>
+      <c r="D2" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1"/>

</xml_diff>

<commit_message>
Added covid msgs to infant child form (#132)
Covid protocol changes to infant_child, pregnancy, and postpartum, and correctly displaying child danger sign at referral follow up
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -15,15 +15,33 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="295">
   <si>
+    <t>form_title</t>
+  </si>
+  <si>
+    <t>form_id</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>instance_name</t>
+  </si>
+  <si>
+    <t>Referral Follow-up</t>
+  </si>
+  <si>
     <t>list_name</t>
   </si>
   <si>
     <t>type</t>
   </si>
   <si>
-    <t>form_title</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -33,51 +51,87 @@
     <t>label::sw</t>
   </si>
   <si>
-    <t>form_id</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>path</t>
+    <t>required</t>
+  </si>
+  <si>
+    <t>relevant</t>
+  </si>
+  <si>
+    <t>appearance</t>
+  </si>
+  <si>
+    <t>read_only</t>
+  </si>
+  <si>
+    <t>constraint</t>
+  </si>
+  <si>
+    <t>constraint_message::en</t>
+  </si>
+  <si>
+    <t>constraint_message::sw</t>
+  </si>
+  <si>
+    <t>calculation</t>
+  </si>
+  <si>
+    <t>choice_filter</t>
+  </si>
+  <si>
+    <t>hint::en</t>
+  </si>
+  <si>
+    <t>hint::sw</t>
   </si>
   <si>
     <t>yes_no</t>
   </si>
   <si>
+    <t>default</t>
+  </si>
+  <si>
+    <t>repeat_count</t>
+  </si>
+  <si>
     <t>yes</t>
   </si>
   <si>
+    <t>referral_follow_up</t>
+  </si>
+  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>instance_name</t>
-  </si>
-  <si>
     <t>Ndiyo</t>
   </si>
   <si>
+    <t>begin group</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>NO_LABEL</t>
+  </si>
+  <si>
+    <t>./source = 'user'</t>
+  </si>
+  <si>
     <t>no</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
+    <t>pages</t>
+  </si>
+  <si>
     <t>Hapana</t>
   </si>
   <si>
-    <t>Referral Follow-up</t>
-  </si>
-  <si>
     <t>reason_didnt_go</t>
   </si>
   <si>
-    <t>referral_follow_up</t>
-  </si>
-  <si>
     <t>no_money</t>
   </si>
   <si>
@@ -93,9 +147,21 @@
     <t>I did not want to go</t>
   </si>
   <si>
+    <t>hidden</t>
+  </si>
+  <si>
     <t>Sikutaka kwenda</t>
   </si>
   <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>source_form</t>
+  </si>
+  <si>
     <t>no_permission</t>
   </si>
   <si>
@@ -105,78 +171,39 @@
     <t>Sikupewa ruhusa ya kwenda</t>
   </si>
   <si>
+    <t xml:space="preserve">string </t>
+  </si>
+  <si>
     <t>other</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
     <t>Other</t>
   </si>
   <si>
-    <t>relevant</t>
-  </si>
-  <si>
     <t>Nyenginezo</t>
   </si>
   <si>
-    <t>appearance</t>
-  </si>
-  <si>
-    <t>read_only</t>
+    <t>original_source_form</t>
   </si>
   <si>
     <t>reason_didnt_get_svc</t>
   </si>
   <si>
-    <t>constraint</t>
-  </si>
-  <si>
-    <t>constraint_message::en</t>
-  </si>
-  <si>
-    <t>constraint_message::sw</t>
-  </si>
-  <si>
-    <t>calculation</t>
-  </si>
-  <si>
-    <t>choice_filter</t>
-  </si>
-  <si>
-    <t>hint::en</t>
-  </si>
-  <si>
-    <t>hint::sw</t>
-  </si>
-  <si>
-    <t>default</t>
-  </si>
-  <si>
-    <t>repeat_count</t>
-  </si>
-  <si>
-    <t>begin group</t>
-  </si>
-  <si>
-    <t>inputs</t>
-  </si>
-  <si>
-    <t>NO_LABEL</t>
-  </si>
-  <si>
-    <t>./source = 'user'</t>
-  </si>
-  <si>
     <t>too_many_people</t>
   </si>
   <si>
+    <t>source_id</t>
+  </si>
+  <si>
     <t>There were too many people</t>
   </si>
   <si>
     <t>Kulikuwa na watu wengi</t>
   </si>
   <si>
+    <t>last_visit_date</t>
+  </si>
+  <si>
     <t>services_not_offered</t>
   </si>
   <si>
@@ -186,15 +213,24 @@
     <t>Huduma nilizotaka hazikuwepo.</t>
   </si>
   <si>
+    <t>refer_flag_small_baby</t>
+  </si>
+  <si>
     <t>no_service_provider_available</t>
   </si>
   <si>
+    <t>refer_neonatal_danger_sign_flag</t>
+  </si>
+  <si>
     <t>No service providers were available</t>
   </si>
   <si>
     <t>Hakukuwa na mtoa huduma</t>
   </si>
   <si>
+    <t>refer_secondary_neonatal_danger_sign_flag</t>
+  </si>
+  <si>
     <t>was_asked_to_pay</t>
   </si>
   <si>
@@ -204,55 +240,19 @@
     <t>Walitaka nilipie huduma</t>
   </si>
   <si>
+    <t>refer_child_danger_sign_flag</t>
+  </si>
+  <si>
     <t>was_treated_badly</t>
   </si>
   <si>
+    <t>refer_child_other_danger_sign_flag</t>
+  </si>
+  <si>
     <t>Health workers treated me badly</t>
   </si>
   <si>
     <t>Wahudumu wa afya hawakunihudumia vizuri</t>
-  </si>
-  <si>
-    <t>pages</t>
-  </si>
-  <si>
-    <t>hidden</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>source_form</t>
-  </si>
-  <si>
-    <t xml:space="preserve">string </t>
-  </si>
-  <si>
-    <t>original_source_form</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>source_id</t>
-  </si>
-  <si>
-    <t>last_visit_date</t>
-  </si>
-  <si>
-    <t>refer_flag_small_baby</t>
-  </si>
-  <si>
-    <t>refer_neonatal_danger_sign_flag</t>
-  </si>
-  <si>
-    <t>refer_secondary_neonatal_danger_sign_flag</t>
-  </si>
-  <si>
-    <t>refer_child_danger_sign_flag</t>
-  </si>
-  <si>
-    <t>refer_child_other_danger_sign_flag</t>
   </si>
   <si>
     <t>refer_muac_flag</t>
@@ -991,15 +991,15 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1074,345 +1074,345 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="F2" s="5" t="s">
-        <v>50</v>
+      <c r="F2" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D3" s="2"/>
       <c r="G3" s="2"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>49</v>
+      <c r="A4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D4" s="2"/>
       <c r="G4" s="2"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D5" s="2"/>
       <c r="G5" s="2"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="3" t="s">
-        <v>68</v>
+      <c r="A9" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>49</v>
+      <c r="A11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>81</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D13" s="2"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>82</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>85</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="3" t="s">
+      <c r="A18" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>49</v>
+      <c r="C18" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="3" t="s">
+      <c r="A19" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>49</v>
+      <c r="C19" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D19" s="2"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="3" t="s">
+      <c r="A20" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>49</v>
+      <c r="C20" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="3" t="s">
+      <c r="A21" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>49</v>
+      <c r="C21" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="A22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>49</v>
+      <c r="C22" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D22" s="2"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B23" s="3" t="s">
+      <c r="A23" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>49</v>
+      <c r="C23" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="D23" s="2"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>92</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>93</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>95</v>
@@ -1436,10 +1436,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>97</v>
@@ -1458,13 +1458,13 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D29" s="2"/>
     </row>
@@ -1476,7 +1476,7 @@
         <v>101</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D30" s="2"/>
       <c r="G30" s="2" t="s">
@@ -1485,37 +1485,37 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>103</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D32" s="2"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D33" s="2"/>
     </row>
@@ -1534,7 +1534,7 @@
         <v>98</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1566,15 +1566,15 @@
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="6" t="s">
         <v>110</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
-      <c r="L38" s="3" t="s">
+      <c r="L38" s="6" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1621,8 +1621,8 @@
       <c r="A42" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>75</v>
+      <c r="B42" s="6" t="s">
+        <v>66</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -1635,7 +1635,7 @@
         <v>105</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -1648,11 +1648,11 @@
         <v>105</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
-      <c r="L44" s="3" t="s">
+      <c r="L44" s="6" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
         <v>105</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -1670,15 +1670,15 @@
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B46" s="3" t="s">
-        <v>79</v>
+      <c r="B46" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
-      <c r="L46" s="3" t="s">
+      <c r="L46" s="6" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1761,49 +1761,49 @@
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="6" t="s">
         <v>130</v>
       </c>
       <c r="C53" s="8"/>
       <c r="D53" s="9"/>
-      <c r="L53" s="3" t="s">
+      <c r="L53" s="6" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
-      <c r="L54" s="3" t="s">
+      <c r="L54" s="6" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="6" t="s">
         <v>133</v>
       </c>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
-      <c r="L55" s="3" t="s">
+      <c r="L55" s="6" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="B56" s="6" t="s">
         <v>86</v>
       </c>
       <c r="C56" s="8"/>
@@ -1813,10 +1813,10 @@
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C57" s="8"/>
@@ -1826,10 +1826,10 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="6" t="s">
         <v>88</v>
       </c>
       <c r="C58" s="8"/>
@@ -1839,10 +1839,10 @@
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="6" t="s">
         <v>89</v>
       </c>
       <c r="C59" s="8"/>
@@ -1852,10 +1852,10 @@
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="3" t="s">
+      <c r="A60" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B60" s="6" t="s">
         <v>90</v>
       </c>
       <c r="C60" s="8"/>
@@ -1865,10 +1865,10 @@
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="6" t="s">
         <v>91</v>
       </c>
       <c r="C61" s="8"/>
@@ -1878,10 +1878,10 @@
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="6" t="s">
         <v>141</v>
       </c>
       <c r="C62" s="8"/>
@@ -1891,10 +1891,10 @@
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" s="6" t="s">
         <v>143</v>
       </c>
       <c r="C63" s="8"/>
@@ -1904,10 +1904,10 @@
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B64" s="6" t="s">
         <v>145</v>
       </c>
       <c r="C64" s="8"/>
@@ -1917,7 +1917,7 @@
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B65" s="13" t="s">
@@ -1930,7 +1930,7 @@
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="3" t="s">
+      <c r="A66" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B66" s="14" t="s">
@@ -1943,7 +1943,7 @@
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B67" s="14" t="s">
@@ -1956,7 +1956,7 @@
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="3" t="s">
+      <c r="A68" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B68" s="14" t="s">
@@ -1969,7 +1969,7 @@
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="3" t="s">
+      <c r="A69" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B69" s="14" t="s">
@@ -2065,10 +2065,10 @@
       <c r="S72" s="19"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B73" s="3" t="s">
+      <c r="A73" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B73" s="6" t="s">
         <v>166</v>
       </c>
       <c r="C73" s="8" t="s">
@@ -2077,71 +2077,71 @@
       <c r="D73" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="G73" s="3" t="s">
+      <c r="G73" s="6" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="3" t="s">
+      <c r="A74" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="B74" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="D74" s="6" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="3" t="s">
+      <c r="A75" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="B75" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D75" s="3" t="s">
+      <c r="D75" s="6" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="3" t="s">
+      <c r="A76" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="D76" s="6" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="3" t="s">
+      <c r="A77" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="B77" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="D77" s="6" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="3" t="s">
+      <c r="A78" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B78" s="6" t="s">
         <v>166</v>
       </c>
       <c r="C78" s="2"/>
@@ -2149,10 +2149,10 @@
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>182</v>
@@ -2160,7 +2160,7 @@
       <c r="D79" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="G79" s="6" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       <c r="D81" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="3" t="s">
+      <c r="F81" s="6" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2213,19 +2213,19 @@
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="3" t="s">
+      <c r="A83" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B83" s="3" t="s">
+      <c r="B83" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C83" s="3" t="s">
+      <c r="C83" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="D83" s="3" t="s">
+      <c r="D83" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="F83" s="3" t="s">
+      <c r="F83" s="6" t="s">
         <v>198</v>
       </c>
     </row>
@@ -2247,19 +2247,19 @@
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="3" t="s">
+      <c r="A85" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B85" s="3" t="s">
+      <c r="B85" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="C85" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D85" s="3" t="s">
+      <c r="D85" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="F85" s="3" t="s">
+      <c r="F85" s="6" t="s">
         <v>206</v>
       </c>
     </row>
@@ -2332,92 +2332,92 @@
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="3" t="s">
+      <c r="A90" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="3" t="s">
+      <c r="B90" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="C90" s="5" t="s">
+      <c r="C90" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="D90" s="6" t="s">
         <v>225</v>
       </c>
       <c r="E90" s="2"/>
-      <c r="F90" s="5" t="s">
+      <c r="F90" s="4" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="3" t="s">
+      <c r="A91" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B91" s="3" t="s">
+      <c r="B91" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="C91" s="5" t="s">
+      <c r="C91" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="D91" s="3" t="s">
+      <c r="D91" s="6" t="s">
         <v>229</v>
       </c>
       <c r="E91" s="2"/>
-      <c r="F91" s="3" t="s">
+      <c r="F91" s="6" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="3" t="s">
+      <c r="A92" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B92" s="3" t="s">
+      <c r="B92" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="C92" s="5" t="s">
+      <c r="C92" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="D92" s="5" t="s">
+      <c r="D92" s="4" t="s">
         <v>233</v>
       </c>
       <c r="E92" s="2"/>
-      <c r="F92" s="3" t="s">
+      <c r="F92" s="6" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="3" t="s">
+      <c r="A93" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="B93" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="C93" s="5" t="s">
+      <c r="C93" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="D93" s="5" t="s">
+      <c r="D93" s="4" t="s">
         <v>237</v>
       </c>
       <c r="E93" s="2"/>
-      <c r="F93" s="3" t="s">
+      <c r="F93" s="6" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="3" t="s">
+      <c r="A94" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="B94" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="D94" s="5" t="s">
+      <c r="D94" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E94" s="2"/>
-      <c r="F94" s="5" t="s">
+      <c r="F94" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -2435,18 +2435,18 @@
         <v>246</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B96" s="7" t="s">
         <v>247</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
@@ -2483,7 +2483,7 @@
         <v>254</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F98" s="2"/>
     </row>
@@ -2501,7 +2501,7 @@
         <v>258</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>259</v>
@@ -2538,13 +2538,13 @@
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>263</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
@@ -2557,7 +2557,7 @@
         <v>265</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C103" s="7" t="s">
         <v>266</v>
@@ -2566,7 +2566,7 @@
         <v>267</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
@@ -2596,13 +2596,13 @@
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B106" s="7" t="s">
         <v>271</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
@@ -2624,7 +2624,7 @@
         <v>275</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="108" ht="15.75" customHeight="1">
@@ -2691,7 +2691,7 @@
         <v>98</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
@@ -2700,7 +2700,7 @@
       <c r="A113" t="s">
         <v>105</v>
       </c>
-      <c r="B113" s="3" t="s">
+      <c r="B113" s="6" t="s">
         <v>286</v>
       </c>
       <c r="C113" s="2"/>
@@ -2710,41 +2710,41 @@
       </c>
     </row>
     <row r="114" ht="12.75" customHeight="1">
-      <c r="A114" s="3" t="s">
+      <c r="A114" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B114" s="3" t="s">
+      <c r="B114" s="6" t="s">
         <v>288</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
-      <c r="L114" s="3" t="s">
+      <c r="L114" s="6" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="115" ht="12.75" customHeight="1">
-      <c r="A115" s="3" t="s">
+      <c r="A115" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B115" s="3" t="s">
+      <c r="B115" s="6" t="s">
         <v>290</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" s="2"/>
-      <c r="L115" s="5" t="s">
+      <c r="L115" s="4" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="116" ht="12.75" customHeight="1">
-      <c r="A116" s="3" t="s">
+      <c r="A116" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B116" s="3" t="s">
+      <c r="B116" s="6" t="s">
         <v>292</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
-      <c r="L116" s="3" t="s">
+      <c r="L116" s="6" t="s">
         <v>293</v>
       </c>
     </row>
@@ -6549,184 +6549,184 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="A8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" ht="12.75" customHeight="1">
+      <c r="A9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" ht="12.75" customHeight="1">
+      <c r="A10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" ht="12.75" customHeight="1">
+      <c r="A11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" ht="12.75" customHeight="1">
+      <c r="A12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" ht="12.75" customHeight="1">
+      <c r="A13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="9" ht="12.75" customHeight="1">
-      <c r="A9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D13" t="s">
         <v>55</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" ht="12.75" customHeight="1">
-      <c r="A10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" ht="12.75" customHeight="1">
-      <c r="A12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" ht="12.75" customHeight="1">
-      <c r="A13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1"/>
@@ -7739,39 +7739,39 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="4">
+        <v>27</v>
+      </c>
+      <c r="C2" s="3">
         <v>43584.0</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>72</v>
+      <c r="D2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1"/>

</xml_diff>

<commit_message>
Added new content in referral followup
</commit_message>
<xml_diff>
--- a/forms/app/referral_follow_up.xlsx
+++ b/forms/app/referral_follow_up.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="299">
   <si>
     <t>type</t>
   </si>
@@ -796,6 +796,12 @@
   </si>
   <si>
     <t xml:space="preserve">../inputs/refer_flag_postpartum_danger_signs = 1 or ../inputs/refer_flag_postpartum_other_signs = 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">has_pregnancy_counselling_referral </t>
+  </si>
+  <si>
+    <t>../inputs/refer_flag_emergency_danger_sign  = 1 or ../inputs/refer_flag_pregnancy_issues  = 1 or  ../inputs/refer_flag_pregnancy_complications = 1</t>
   </si>
   <si>
     <t>referral_days</t>
@@ -1082,7 +1088,9 @@
     <col customWidth="1" min="1" max="1" width="40.0"/>
     <col customWidth="1" min="2" max="2" width="43.57"/>
     <col customWidth="1" min="3" max="3" width="37.29"/>
-    <col customWidth="1" min="4" max="17" width="14.43"/>
+    <col customWidth="1" min="4" max="5" width="14.43"/>
+    <col customWidth="1" min="6" max="6" width="91.0"/>
+    <col customWidth="1" min="7" max="17" width="14.43"/>
     <col customWidth="1" min="18" max="26" width="8.71"/>
   </cols>
   <sheetData>
@@ -2827,21 +2835,30 @@
       </c>
     </row>
     <row r="119" ht="12.75" customHeight="1">
-      <c r="A119" s="1" t="s">
+      <c r="A119" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B119" s="1" t="s">
+      <c r="B119" s="3" t="s">
         <v>252</v>
       </c>
       <c r="C119" s="1"/>
       <c r="D119" s="1"/>
-      <c r="L119">
-        <v>3.0</v>
+      <c r="L119" s="3" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="120" ht="12.75" customHeight="1">
+      <c r="A120" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>254</v>
+      </c>
       <c r="C120" s="1"/>
       <c r="D120" s="1"/>
+      <c r="L120">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="121" ht="12.75" customHeight="1">
       <c r="C121" s="1"/>
@@ -6602,6 +6619,10 @@
     <row r="1060" ht="12.75" customHeight="1">
       <c r="C1060" s="1"/>
       <c r="D1060" s="1"/>
+    </row>
+    <row r="1061" ht="12.75" customHeight="1">
+      <c r="C1061" s="1"/>
+      <c r="D1061" s="1"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -6627,7 +6648,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B1" s="19" t="s">
         <v>1</v>
@@ -6641,30 +6662,30 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>203</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -6672,13 +6693,13 @@
         <v>223</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D4" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -6686,13 +6707,13 @@
         <v>223</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -6700,13 +6721,13 @@
         <v>223</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -6714,97 +6735,97 @@
         <v>223</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D7" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>270</v>
-      </c>
       <c r="D13" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1"/>
@@ -7817,27 +7838,27 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B2" t="s">
         <v>137</v>
@@ -7846,10 +7867,10 @@
         <v>43584.0</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1"/>

</xml_diff>